<commit_message>
Simplify TCS/TDS to 4 vouchers with combined month netting
- Only vouchers 41-44 for TCS/TDS (prepaid/postpaid x tcs/tds)
- Include current and prior month rows in the same vouchers
- Same sign rule for all months: negative net -> debit, positive -> credit
- Net amounts at state level per TCS/TDS column before posting

Co-authored-by: shrikant2891 <shrikant2891@gmail.com>
</commit_message>
<xml_diff>
--- a/MP Summary.xlsx
+++ b/MP Summary.xlsx
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" style="2" min="1" max="1"/>
@@ -800,71 +800,64 @@
     <row r="15">
       <c r="A15" s="25" t="inlineStr">
         <is>
-          <t>41-44  TCS / TDS receivable (current month) by prepaid &amp; postpaid</t>
+          <t>41-44  TCS / TDS receivable by prepaid &amp; postpaid (current + prior month)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="25" t="inlineStr">
-        <is>
-          <t>45-48  TCS / TDS payable (prior month) by prepaid &amp; postpaid</t>
-        </is>
-      </c>
+      <c r="A16" s="25" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="25" t="inlineStr"/>
+      <c r="A17" s="26" t="inlineStr">
+        <is>
+          <t>Posting rules</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="26" t="inlineStr">
-        <is>
-          <t>Posting rules</t>
+      <c r="A18" s="25" t="inlineStr">
+        <is>
+          <t>Expense &amp; GST lines use state_code_to at state level.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="25" t="inlineStr">
         <is>
-          <t>Expense &amp; GST lines use state_code_to at state level.</t>
+          <t>TCS / TDS lines use tcs_state_code_to, net at state level, and include current + prior month.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="25" t="inlineStr">
         <is>
-          <t>TCS / TDS lines use tcs_state_code_to and net at state level.</t>
+          <t>TCS/TDS: negative net -&gt; debit receivable; positive net -&gt; credit receivable.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="25" t="inlineStr">
         <is>
-          <t>TCS/TDS current month: negative net -&gt; debit receivable; prior month: negative net -&gt; credit payable.</t>
+          <t>IGST input: IN-DL -&gt; 142067; other states -&gt; 142013.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="25" t="inlineStr">
         <is>
-          <t>IGST input: IN-DL -&gt; 142067; other states -&gt; 142013.</t>
+          <t>Debtor &amp; provision ledgers always use IN-OTH.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="25" t="inlineStr">
         <is>
-          <t>Debtor &amp; provision ledgers always use IN-OTH.</t>
+          <t>Negative Summary values -&gt; Debit expense/GST, Credit debtor.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="25" t="inlineStr">
-        <is>
-          <t>Negative Summary values -&gt; Debit expense/GST, Credit debtor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="25" t="inlineStr">
         <is>
           <t>OI opening vouchers reverse the prior-month OI expense entries.</t>
         </is>
@@ -881,7 +874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1106,46 +1099,6 @@
       </c>
       <c r="B21" t="n">
         <v>44</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>TCS_POSTPAID_PRIOR</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>TDS_POSTPAID_PRIOR</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>TCS_PREPAID_PRIOR</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>TDS_PREPAID_PRIOR</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix TCS/TDS state fallback and month inclusion
- Use state_code_to when tcs_state_code_to is NA so prior-month rows post
- Include latest two Summary months with normalized month labels
- Net TCS/TDS at state level per GL to prevent duplicate state lines
- Mirror fixes in VBA macro (MonthLabelFromCell, TcsTdsState, gl|state agg)

Co-authored-by: shrikant2891 <shrikant2891@gmail.com>
</commit_message>
<xml_diff>
--- a/MP Summary.xlsx
+++ b/MP Summary.xlsx
@@ -824,7 +824,7 @@
     <row r="19">
       <c r="A19" s="25" t="inlineStr">
         <is>
-          <t>TCS / TDS lines use tcs_state_code_to, net at state level, and include current + prior month.</t>
+          <t>TCS / TDS lines use tcs_state_code_to (fallback state_code_to), net at state level per GL, and include the latest two Summary months.</t>
         </is>
       </c>
     </row>
@@ -3666,7 +3666,7 @@
         </is>
       </c>
       <c r="J41" s="33" t="n">
-        <v>302</v>
+        <v>604</v>
       </c>
       <c r="K41" s="33" t="n">
         <v>0</v>
@@ -3826,7 +3826,7 @@
         </is>
       </c>
       <c r="B44" s="31" t="n">
-        <v>142016</v>
+        <v>142015</v>
       </c>
       <c r="C44" s="36" t="n">
         <v>46234</v>
@@ -3852,7 +3852,7 @@
         </is>
       </c>
       <c r="J44" s="33" t="n">
-        <v>105.51</v>
+        <v>1898.55</v>
       </c>
       <c r="K44" s="33" t="n">
         <v>0</v>
@@ -3888,7 +3888,7 @@
         </is>
       </c>
       <c r="B45" s="31" t="n">
-        <v>142015</v>
+        <v>142016</v>
       </c>
       <c r="C45" s="36" t="n">
         <v>46234</v>
@@ -3914,7 +3914,7 @@
         </is>
       </c>
       <c r="J45" s="33" t="n">
-        <v>1898.55</v>
+        <v>105.51</v>
       </c>
       <c r="K45" s="33" t="n">
         <v>0</v>
@@ -4413,7 +4413,7 @@
         <v>0</v>
       </c>
       <c r="K53" s="33" t="n">
-        <v>3329.2</v>
+        <v>3631.2</v>
       </c>
       <c r="L53" s="31" t="inlineStr">
         <is>
@@ -5066,7 +5066,7 @@
         </is>
       </c>
       <c r="B64" s="31" t="n">
-        <v>142016</v>
+        <v>142015</v>
       </c>
       <c r="C64" s="36" t="n">
         <v>46234</v>
@@ -5092,7 +5092,7 @@
         </is>
       </c>
       <c r="J64" s="33" t="n">
-        <v>0.12</v>
+        <v>0.25</v>
       </c>
       <c r="K64" s="33" t="n">
         <v>0</v>
@@ -5128,7 +5128,7 @@
         </is>
       </c>
       <c r="B65" s="31" t="n">
-        <v>142015</v>
+        <v>142016</v>
       </c>
       <c r="C65" s="36" t="n">
         <v>46234</v>
@@ -5154,7 +5154,7 @@
         </is>
       </c>
       <c r="J65" s="33" t="n">
-        <v>0.25</v>
+        <v>0.12</v>
       </c>
       <c r="K65" s="33" t="n">
         <v>0</v>
@@ -5500,7 +5500,7 @@
         </is>
       </c>
       <c r="B71" s="31" t="n">
-        <v>142016</v>
+        <v>142015</v>
       </c>
       <c r="C71" s="36" t="n">
         <v>46234</v>
@@ -5526,7 +5526,7 @@
         </is>
       </c>
       <c r="J71" s="33" t="n">
-        <v>0.25</v>
+        <v>0.18</v>
       </c>
       <c r="K71" s="33" t="n">
         <v>0</v>
@@ -5562,7 +5562,7 @@
         </is>
       </c>
       <c r="B72" s="31" t="n">
-        <v>142015</v>
+        <v>142016</v>
       </c>
       <c r="C72" s="36" t="n">
         <v>46234</v>
@@ -5588,7 +5588,7 @@
         </is>
       </c>
       <c r="J72" s="33" t="n">
-        <v>0.18</v>
+        <v>0.25</v>
       </c>
       <c r="K72" s="33" t="n">
         <v>0</v>
@@ -5748,7 +5748,7 @@
         </is>
       </c>
       <c r="B75" s="31" t="n">
-        <v>142016</v>
+        <v>142015</v>
       </c>
       <c r="C75" s="36" t="n">
         <v>46234</v>
@@ -5810,7 +5810,7 @@
         </is>
       </c>
       <c r="B76" s="31" t="n">
-        <v>142015</v>
+        <v>142016</v>
       </c>
       <c r="C76" s="36" t="n">
         <v>46234</v>
@@ -12664,13 +12664,13 @@
         </is>
       </c>
       <c r="C10" s="34" t="n">
-        <v>3329.2</v>
+        <v>3631.2</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>3329.2</v>
+        <v>3631.2</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">

</xml_diff>